<commit_message>
Record McMaster plus-5 on batch 721 and refresh the 9/18 sheet.
Entered leftover invoices 72068812/10143 (over-PPV Transfer AP 375),
72087570/10144, 72012111/10145, 72013304/10146, and 71839575/10147
(missing_receipt Ruben HOLDs). First five left alone. Sheet now has
all 10 rows.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -936,8 +936,403 @@
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>72068812</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>58221</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>336.49</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='@Shawn McKibben HOLD (price-does-not-match) on McMaster-Carr 72068812 PO 58221 PDF $336.49. Leftover vs invoice line is over the PPV gate. Receipts were NOT selected so purchasing can unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI.' @mention=Comments persisted @Shawn McKibben. No mention/notify field on the record. Dedicated GET comments/mentions/notifications → [{'suffix': 'comments', 'http': 404}, {'suffix': 'mentions', 'http': 404}, {'suffix': 'notifications', 'http': 404}]. @mention notify not confirmed — cannot claim a user alert fired..</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>10143</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>72087570</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>59235</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>30.32</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59235 for McMaster invoice #72087570. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>10144</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 12.29</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>72012111</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>59219</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>217.39</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59219 for McMaster invoice #72012111. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>10145</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 30.59</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>72013304</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>58221</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>443.49</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58221 for McMaster invoice #72013304. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>10146</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 18.45</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>71839575</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>59191</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>217.39</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59191 for McMaster invoice #71839575. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Ruben Perez</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>10147</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 30.59</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q6"/>
+  <autoFilter ref="A1:Q11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -974,7 +1369,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -984,7 +1379,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Write over-PPV @Shawn notes to the Comments tab, not the header string.
Kyle confirmed 10140 was on Transfer AP but the Comments tab was empty.
The UI list is lists.Comments_1 (HtmlValue + Entity 203 + FormId 218).
Backfilled 10140 item 884 and 10143 item 886. Header Comments is ignored
and is never reported as persisted (NOTE-43).

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -738,7 +738,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='@Shawn McKibben HOLD (price-does-not-match) on McMaster-Carr 71001379 PO 59069 PDF $85.82. Leftover vs invoice line is over the PPV gate. Receipts were NOT selected so purchasing can unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI.' @mention=Comments persisted @Shawn McKibben. No mention/notify field on the record. Dedicated GET comments/mentions/notifications → [{'suffix': 'comments', 'http': 404}, {'suffix': 'mentions', 'http': 404}, {'suffix': 'notifications', 'http': 404}]. @mention notify not confirmed — cannot claim a user alert fired..</t>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='@Shawn McKibben HOLD (price-does-not-match) on McMaster-Carr 71001379 PO 59069 PDF $85.82. Leftover vs invoice line is over the PPV gate. Receipts were NOT selected so purchasing can unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI.'. Comments tab persisted @Shawn McKibben (list Comments_1 item 884, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='@Shawn McKibben HOLD (price-does-not-match) on McMaster-Carr 72068812 PO 58221 PDF $336.49. Leftover vs invoice line is over the PPV gate. Receipts were NOT selected so purchasing can unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI.' @mention=Comments persisted @Shawn McKibben. No mention/notify field on the record. Dedicated GET comments/mentions/notifications → [{'suffix': 'comments', 'http': 404}, {'suffix': 'mentions', 'http': 404}, {'suffix': 'notifications', 'http': 404}]. @mention notify not confirmed — cannot claim a user alert fired..</t>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='@Shawn McKibben HOLD (price-does-not-match) on McMaster-Carr 72068812 PO 58221 PDF $336.49. Leftover vs invoice line is over the PPV gate. Receipts were NOT selected so purchasing can unreceive, change the PO price, and re-receive. Do not alter receipt unit price in GI.'. Comments tab persisted @Shawn McKibben (list Comments_1 item 886, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Record McMaster receipt-retry results and leave unfinished HOLDs alone.
Finished 10144/10145/10147. 10139 Select Receipts 400 on locked 24247;
10142 only one of four PDF lines received (bogus PPV removed); 10146
PO 58221 leftovers are AQPC, not McMaster 4082T15.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -659,7 +659,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59056 for McMaster invoice #71080498. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): open leftover 24247 is 18@20.72 on PO 59056 (PDF 9565K38 18@20.72) but Select Receipts PUT returned 400 'items in this list are not valid'. Receipt 24247 is locked / Quantity_Remaining 0. Do not first-open 23841 (unreceived via 24246). Do not invent Success. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59224 for McMaster invoice #72094446. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): PDF has four merch lines (3616N12 6@7.00, 2151A27 1@23.18, 5513T12 1@6.32, 93320A385 2@17.56) + Shipping 24.59 = $131.21. Only leftover on PO 59224 is 24248 1@17.56 (line 04). Selected that one receipt. Do not first-open guess the missing three lines / second spacer. Incorrect in-gate PPV $5.62 was posted then Removed (GET-proved gone). Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1039,26 +1039,18 @@
       <c r="E8" s="2" t="n">
         <v>30.32</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59235 for McMaster invoice #72087570. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59235. Select Receipts 24249 3@6.01 on PO 59235. Invoice #=72087570 (exact PDF, not subject Order #). Fees=Shipping 12.29 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24249] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
         <v>10144</v>
       </c>
@@ -1089,7 +1081,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
@@ -1118,26 +1110,18 @@
       <c r="E9" s="2" t="n">
         <v>217.39</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59219 for McMaster invoice #72012111. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59219. Select Receipts 24244 40@4.67 on PO 59219. Invoice #=72012111 (exact PDF, not subject Order #). Fees=Shipping 30.59 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24244] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
         <v>10145</v>
       </c>
@@ -1168,7 +1152,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr"/>
@@ -1204,7 +1188,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 58221 for McMaster invoice #72013304. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): PDF 4082T15 24@17.71 + Shipping 18.45 = $443.49 on PO 58221. Open leftovers on 58221 are AQPC June lines at $15–$50 (20397–20404), not McMaster 4082T15. Do not first-open guess. Flag status=entered-with-issues.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1276,26 +1260,18 @@
       <c r="E11" s="2" t="n">
         <v>217.39</v>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): no open receipt leftover on PO 59191 for McMaster invoice #71839575. Do not first-open guess. @Ruben Perez: receiving must receive the PO so AP can Select Receipts. Outlook Entered with issues. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59191. Select Receipts 24245 40@4.67 on PO 59191. Invoice #=71839575 (exact PDF, not subject Order #). Fees=Shipping 30.59 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[{'id': 24245, 'qty': 40.0}] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
         <v>10147</v>
       </c>
@@ -1326,7 +1302,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
@@ -1369,7 +1345,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Encode NOTE-44: Fees are not missing merch receipt lines.
Do not HOLD missing_receipt when leftover PDF dollars are Additional
Charge Fees id 11 (posted or to-be-posted). McMaster 10147/10144/10145
are Success; leave 10142 as real missing merch.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=59235. Select Receipts 24249 3@6.01 on PO 59235. Invoice #=72087570 (exact PDF, not subject Order #). Fees=Shipping 12.29 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24249] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59235. Select Receipts 24249 3@6.01 on PO 59235. Invoice #=72087570 (exact PDF, not subject Order #). Fees=Shipping 12.29 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Posted=30.32 matches PDF (merch 18.03 + Fees 12.29). Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=59219. Select Receipts 24244 40@4.67 on PO 59219. Invoice #=72012111 (exact PDF, not subject Order #). Fees=Shipping 30.59 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24244] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59219. Select Receipts 24244 40@4.67 on PO 59219. Invoice #=72012111 (exact PDF, not subject Order #). Fees=Shipping 30.59 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Posted=217.39 matches PDF (merch 186.80 + Fees 30.59). Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=59191. Select Receipts 24245 40@4.67 on PO 59191. Invoice #=71839575 (exact PDF, not subject Order #). Fees=Shipping 30.59 (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[{'id': 24245, 'qty': 40.0}] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59191. Select Receipts 24245 40@4.67 on PO 59191. Invoice #=71839575 (exact PDF, not subject Order #). Fees=Shipping 30.59 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Posted=217.39 matches PDF (merch 186.80 + Fees 30.59). Kyle 2026-09-21: Validate Invoice passed in live UI (Invoice_Validation GET is always null — NOTE-41). Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Record McMaster plus-5 on batch 721 and lock the new header ids.
10149/10150/10151 finished. 10148 over-PPV moved to Transfer AP with
Comments_1 @Shawn. 10152 missing_receipt stayed on 721 with @Shawn.
Leave 10138-10147 unchanged.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1307,8 +1307,379 @@
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>71743140</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>59159</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>35.85</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='Comments tab persisted @Shawn McKibben (list Comments_1 item 887, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.' @mention=Comments tab persisted @Shawn McKibben (list Comments_1 item 887, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored..</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>10148</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 13.61</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>71740547</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>59120</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>151.44</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59120. Select Receipts 23997 5@29.25 on PO 59120. Invoice #=71740547 (exact PDF, not subject Order #). Fees=Shipping 5.19 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[23997] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="n">
+        <v>10149</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 5.19</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>71642803</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>59159</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>186.22</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59159. Select Receipts 24234 1@32.28; 24235 6@17.6; 24236 6@2.91; 24237 1@11.2; 24238 1@6.17 on PO 59159. Invoice #=71642803 (exact PDF, not subject Order #). Fees=Shipping 13.51 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24234, 24235, 24236, 24237, 24238] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n">
+        <v>10150</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 13.51</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>71668723</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>59120</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>5832.28</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59120. Select Receipts 24000 20@63.93; 24008 5@129.16; 24009 10@7.49; 24010 15@59.77; 24011 1@25.25; 23995 5@46.81; 24012 5@47.04; 24013 5@35.28; 24014 4@16.02; 24015 2@12.51; 24016 2@8.75; 24001 5@43.98; 24017 1@30.95; 24018 2@16.61; 24019 8@10.1; 23996 4@8.35; 24020 10@1.84; 24022 5@5.24; 24023 2@4.58; 24024 3@4.66; 23994 10@19.05; 23999 10@19.05; 24002 5@103.9; 23998 2@29.25; 23997 5@29.25; 24003 10@21.67; 24004 20@3.37; 24005 10@8.35; 24006 1@14.75; 24007 1@37.25 on PO 59120. Invoice #=71668723 (exact PDF, not subject Order #). Fees=Shipping 203.89 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=-35.82. Attach status=attached. Finish Select Receipts selected ids=[24000, 24001, 24002, 23997, 24003, 24004, 24005, 24006, 24007, 24008, 24009, 24010, 24011, 23995, 24012, 24013, 24014, 24015, 24016, 24017, 24018, 24019, 23996, 24020, 24022, 24023, 24024, 23994, 23999, 23998] fees=already-posted ppv=posted. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
+        <v>10151</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 203.89</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>-35.82</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>71401129</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>59125</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>257.72</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Shawn McKibben. HOLD (receipt): no open receipt leftover on PO 59125 for McMaster invoice #71401129. Do not first-open guess. @Shawn McKibben: receiving must receive the PO so AP can Select Receipts. Comments_1 @Shawn (NOTE-45). Do not Transfer AP. Finish Select Receipts blocked-400 ids=[23939, 23940, 23941] fees=already-posted ppv=none. Outlook Entered with issues. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted @Shawn McKibben (list Comments_1 item 888, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False batch_still=API Agent - 9/18/26 McMaster mail_send=False.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>10152</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 14.6</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q11"/>
+  <autoFilter ref="A1:Q16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1345,7 +1716,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1355,7 +1726,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record McMaster plus-15 on batch 721 and lock the new header ids.
Entered 71254641/10153, 71236251/10154, 71183051/10155, 71098307/10156,
70907154/10157. Four Success (Select Receipts + Fees, amount=PDF) and
10154 over-PPV Transfer AP + Comments_1 @Shawn 104. Leave 10138-10152
untouched; leftover after cap is 70759737/59014 and 70758802/59001.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1678,8 +1678,371 @@
       </c>
       <c r="Q16" s="2" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>71254641</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>59103</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>931.89</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59103. Select Receipts 23835 10@63.34; 23836 5@23.64; 23837 1@11.27; 23838 4@4.95; 23839 2@65.88 on PO 59103. Invoice #=71254641 (exact PDF, not subject Order #). Fees=Shipping 17.46 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[23835, 23836, 23837, 23838, 23839] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
+        <v>10153</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 17.46</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>71236251</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>59103</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>91.25</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='Comments tab persisted @Shawn McKibben (list Comments_1 item 889, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.' @mention=Comments tab persisted @Shawn McKibben (list Comments_1 item 889, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored..</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>10154</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 13.07</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>71183051</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>59089</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>191.43</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59089. Select Receipts 23783 8@2.2; 23792 1@44.53; 23784 12@1.21; 23785 6@1.88; 23786 1@5.67; 23787 2@15.88; 23788 2@18.52; 23789 2@2.68; 23790 2@2.52; 23791 2@2.05 on PO 59089. Invoice #=71183051 (exact PDF, not subject Order #). Fees=Shipping 14.53 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[23783, 23784, 23785, 23786, 23787, 23788, 23789, 23790, 23791, 23792] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
+        <v>10155</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 14.53</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>71098307</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>59078</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>82.56999999999999</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59078. Select Receipts 23701 4@8.1; 23702 4@8.91 on PO 59078. Invoice #=71098307 (exact PDF, not subject Order #). Fees=Shipping 14.53 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[23701, 23702] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
+        <v>10156</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 14.53</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>70907154</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>59046</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>123.78</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59046. Select Receipts 23826 6@14.52; 23827 1@7.53; 23828 1@9.01; 23829 1@5.74 on PO 59046. Invoice #=70907154 (exact PDF, not subject Order #). Fees=Shipping 14.38 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[23826, 23827, 23828, 23829] fees=already-posted ppv=none. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n">
+        <v>10157</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 14.38</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>entered-in-ai</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q16"/>
+  <autoFilter ref="A1:Q21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1726,7 +2089,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record McMaster plus-20 on batch 721 and lock the new header ids.
Entered 70759737/10158 (missing_receipt HOLD on 721, Comments_1 @Shawn 104)
and 70758802/10159 (over-PPV Transfer AP + Comments_1 @Shawn). Inbox after
Aug 1 was exhausted at 2 new bills. Leave 10138-10157 untouched.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exception counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$Q$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2041,8 +2041,166 @@
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>70759737</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>59014</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1037.59</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>category=missing_receipt; owner=Shawn McKibben. HOLD (receipt): no open receipt leftover on PO 59014 for McMaster invoice #70759737. Do not first-open guess. @Shawn McKibben: receiving must receive the PO so AP can Select Receipts. Comments_1 @Shawn (NOTE-45). Do not Transfer AP. Outlook Entered with issues. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted @Shawn McKibben (list Comments_1 item 891, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False batch_still=API Agent - 9/18/26 McMaster mail_send=False.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>missing_receipt</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>10158</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/18/26 McMaster (721)</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 34.39</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr Supply Company</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>70758802</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>59001</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>49.19</v>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>category=price_variance; owner=Shawn McKibben. HOLD (price-does-not-match): leftover vs invoice line is over the PPV gate. Do not Select Receipts on that line. @Shawn McKibben: purchasing must unreceive, change the PO price, and re-receive. Finish Select Receipts selected ids=[23700] fees=already-posted ppv=none. Outlook Entered with issues. Flag status=entered-with-issues. Transfer AP status=moved batch_id=375 comment='Comments tab persisted @Shawn McKibben (list Comments_1 item 892, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.' @mention=Comments tab persisted @Shawn McKibben (list Comments_1 item 892, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored..</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>price_variance</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Shawn McKibben</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>10159</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>TRANSFER AP (375)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Shipping 25.0</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>attached</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>entered-with-issues</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q21"/>
+  <autoFilter ref="A1:Q23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2079,7 +2237,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -2089,7 +2247,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record McMaster 71080498 / 10139 Success on batch 721.
Kyle selected 24247 18@20.72. Shipping posted as Fees id 11 $22.35.
Removed leftover Freight External $22.24 and the offsetting PPV.
Invoice amount and verification both $395.31. Lock 10139 GET-only.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -652,26 +652,18 @@
       <c r="E3" s="2" t="n">
         <v>395.31</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): open leftover 24247 is 18@20.72 on PO 59056 (PDF 9565K38 18@20.72) but Select Receipts PUT returned 400 'items in this list are not valid'. Receipt 24247 is locked / Quantity_Remaining 0. Do not first-open 23841 (unreceived via 24246). Do not invent Success. Flag status=entered-with-issues.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Ruben Perez</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59056. Select Receipts 24247 18@20.72 on PO 59056. Invoice #=71080498 (exact PDF, not subject Order #). Fees=Shipping 22.35 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n">
         <v>10139</v>
       </c>
@@ -702,7 +694,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr"/>
@@ -2233,7 +2225,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>missing_receipt</t>
+          <t>price_variance</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2243,11 +2235,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>price_variance</t>
+          <t>missing_receipt</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record McMaster 71401129 / 10152 Success; lock the header.
Live GET-prove: Type 3 on 721, Amount=Verification=PDF 257.72, receipts
23939-23941, Fees 14.60, PPV -14.60. Move 10152 to do-not-mutate.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -1615,26 +1615,18 @@
       <c r="E16" s="2" t="n">
         <v>257.72</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Shawn McKibben. HOLD (receipt): no open receipt leftover on PO 59125 for McMaster invoice #71401129. Do not first-open guess. @Shawn McKibben: receiving must receive the PO so AP can Select Receipts. Comments_1 @Shawn (NOTE-45). Do not Transfer AP. Finish Select Receipts blocked-400 ids=[23939, 23940, 23941] fees=already-posted ppv=none. Outlook Entered with issues. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted @Shawn McKibben (list Comments_1 item 888, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False batch_still=API Agent - 9/18/26 McMaster mail_send=False.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>missing_receipt</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Shawn McKibben</t>
-        </is>
-      </c>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59125. Select Receipts 23939 8@10.89; 23940 8@8.08; 23941 16@5.71 on PO 59125. Invoice #=71401129 (exact PDF, not subject Order #). Fees=Shipping 14.6 (Additional Charge Fees id 11, not missing merch lines / not PPV). PPV=-14.60. Attach status=attached. Flag status=entered-in-ai.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="n">
         <v>10152</v>
       </c>
@@ -1650,7 +1642,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>-14.60</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1665,7 +1657,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr"/>
@@ -2239,7 +2231,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record Transfer AP + Comments_1 for McMaster 72013304 and 70759737.
Live GET-prove: 10146 and 10158 moved 721 → TRANSFER AP 375. Comments_1
items 925 and 926 @Shawn mention-id 104. No Select. Still HOLD.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-18-mcmaster.xlsx
+++ b/runs/AP-run-2026-09-18-mcmaster.xlsx
@@ -1180,7 +1180,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Ruben Perez. HOLD (receipt): PDF 4082T15 24@17.71 + Shipping 18.45 = $443.49 on PO 58221. Open leftovers on 58221 are AQPC June lines at $15–$50 (20397–20404), not McMaster 4082T15. Do not first-open guess. Flag status=entered-with-issues.</t>
+          <t>category=missing_receipt; owner=Shawn McKibben. HOLD (receipt): Kyle override — move McMaster 72013304 / 10146 from API Agent - 9/18/26 McMaster (721) to Transfer AP. PDF merch=4082T15 24.0@17.71; selected=none. @Shawn McKibben Kyle asked AP to move McMaster-Carr 72013304 / KIMCO 10146 (PDF $443.49, PO 58221) to Transfer AP. Override of missing_receipt-stays-on-721. Type 3 header had receipts=0 fees=Shipping 18.45. PDF merch=4082T15 24.0@17.71. Live PO PO58221-AMERICAN QUALITY POWDERCOATING is AQPC-titled. Open leftovers on 58221 are not McMaster 4082T15. Do not Select those AQPC leftovers (would lock the wrong merch). Receive McMaster 4082T15 qty 24 on the correct PO, or unreceive/reprice/re-receive if the PO line is wrong. Treyce owns Transfer AP follow-through. Do not alter receipt unit price in GI. No email. Transfer AP status=moved batch_id=375 Comments_1 items=[925] mention_id=104 tab=Comments tab persisted @Shawn McKibben (list Comments_1 item 925, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.. mail_send=False.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Ruben Perez</t>
+          <t>Shawn McKibben</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 9/18/26 McMaster (721)</t>
+          <t>TRANSFER AP (375)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>category=missing_receipt; owner=Shawn McKibben. HOLD (receipt): no open receipt leftover on PO 59014 for McMaster invoice #70759737. Do not first-open guess. @Shawn McKibben: receiving must receive the PO so AP can Select Receipts. Comments_1 @Shawn (NOTE-45). Do not Transfer AP. Outlook Entered with issues. Flag status=entered-with-issues. Comments_1 missing_receipt status=added tab=Comments tab persisted @Shawn McKibben (list Comments_1 item 891, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored. transfer_ap=False batch_still=API Agent - 9/18/26 McMaster mail_send=False.</t>
+          <t>category=missing_receipt; owner=Shawn McKibben. HOLD (receipt): Kyle override — move McMaster 70759737 / 10158 from API Agent - 9/18/26 McMaster (721) to Transfer AP. PDF merch=98935A744 12.0@12.1; 6698K17 24.0@21.24; 5909K49 48.0@1.55; 5909K36 24.0@4.47; 5544A25 12.0@11.32; 98410A133 2.0@15.36; selected=none. @Shawn McKibben Kyle asked AP to move McMaster-Carr 70759737 / KIMCO 10158 (PDF $1037.59, PO 59014) to Transfer AP. Override of missing_receipt-stays-on-721. Type 3 header had receipts=0 fees=Shipping 34.39. PDF merch=98935A744 12.0@12.1; 6698K17 24.0@21.24; 5909K49 48.0@1.55; 5909K36 24.0@4.47; 5544A25 12.0@11.32; 98410A133 2.0@15.36. PO PO59014-MCMASTER-CARR has zero open merch leftovers matching the PDF. Receive the PO 59014 lines so AP can Select Receipts. Treyce owns Transfer AP follow-through. Do not alter receipt unit price in GI. No email. Transfer AP status=moved batch_id=375 Comments_1 items=[926] mention_id=104 tab=Comments tab persisted @Shawn McKibben (list Comments_1 item 926, mention-node id 104). User-alert/notify API not confirmed — dedicated GET comments/mentions/notifications are 404. Header Comments string is the wrong surface and is ignored.. mail_send=False.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 9/18/26 McMaster (721)</t>
+          <t>TRANSFER AP (375)</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">

</xml_diff>